<commit_message>
feat: add ID Card Manager Pro with Excel/DB support, GDrive integration, and advanced table filters
Co-authored-by: biswasp87 <76902729+biswasp87@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/uploads/test_data.xlsx
+++ b/uploads/test_data.xlsx
@@ -444,11 +444,7 @@
           <t>Alice</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>S001.jpg</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>